<commit_message>
feat(ui): sincronizar estilizacao da timeline, base Excel atualizada e automacao de build limpo
</commit_message>
<xml_diff>
--- a/Calendario_Digital_Base.xlsx
+++ b/Calendario_Digital_Base.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R249"/>
+  <dimension ref="A1:R250"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10552,7 +10552,7 @@
         <v>0</v>
       </c>
       <c r="Q181">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R181" t="str">
         <v/>
@@ -10655,7 +10655,7 @@
         <v>Sim</v>
       </c>
       <c r="N183" t="str">
-        <v>Cliente Previsto</v>
+        <v>Cliente Confirmado</v>
       </c>
       <c r="O183" t="str">
         <v>2026-09-18</v>
@@ -10664,7 +10664,7 @@
         <v/>
       </c>
       <c r="Q183">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R183" t="str">
         <v/>
@@ -14366,9 +14366,65 @@
         <v/>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>svc-nextcal-1789991888343-p0574</v>
+      </c>
+      <c r="B250">
+        <v>11</v>
+      </c>
+      <c r="C250" t="str">
+        <v>CHI - Grupo CMPC - Envases</v>
+      </c>
+      <c r="D250" t="str">
+        <v/>
+      </c>
+      <c r="E250" t="str">
+        <v/>
+      </c>
+      <c r="F250" t="str">
+        <v/>
+      </c>
+      <c r="G250">
+        <v>0</v>
+      </c>
+      <c r="H250">
+        <v>0</v>
+      </c>
+      <c r="I250">
+        <v>0</v>
+      </c>
+      <c r="J250" t="str">
+        <v>2027-03-15</v>
+      </c>
+      <c r="K250" t="str">
+        <v>2027-03-19</v>
+      </c>
+      <c r="L250" t="str">
+        <v>LF</v>
+      </c>
+      <c r="M250" t="str">
+        <v>Não</v>
+      </c>
+      <c r="N250" t="str">
+        <v>Cliente Previsto</v>
+      </c>
+      <c r="O250" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="P250" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q250">
+        <v>6</v>
+      </c>
+      <c r="R250" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R249"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R250"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>